<commit_message>
Alta de GeTAU (AR) en excluidos tras revisión: civic tech de monitoreo, no entra
- GeTAU (Córdoba): WebApp de IA + geolocalización + participación vecinal para
  monitoreo del arbolado urbano (ONG Acción Ambiental + UNC). Revisión de 2ª
  opinión coincide con el juicio del equipo: la participación es aporte de
  datos (censo colaborativo) y la IA opera sobre los datos de árboles, no
  sobre aportes de un proceso participativo → NO ENTRA (criterio: civic tech
  de reporte/monitoreo; análogo a ParticipACT, dIAra, Pa' que veás).
- Entregable 2 pasa a 80 casos = 12 + 49 + 19; verificadores y handoff (§10)
  actualizados. Entregables 1 y 3 intactos (no afecta ningún cálculo).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgJzdTwpnKB7PvGwYgsS2F
</commit_message>
<xml_diff>
--- a/data/final/Casos_excluidos_ILIA2026.xlsx
+++ b/data/final/Casos_excluidos_ILIA2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Casos excluidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos excluidos'!$A$5:$F$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos excluidos'!$A$5:$F$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total: 79 casos  ·  Base 2025 incluidos→excluidos: 12  ·  Base 2025 exclusión reconfirmada: 49  ·  Nuevos 2026 no incluidos: 18</t>
+          <t>Total: 80 casos  ·  Base 2025 incluidos→excluidos: 12  ·  Base 2025 exclusión reconfirmada: 49  ·  Nuevos 2026 no incluidos: 19</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>BP-Classificador de Propostas (indexação/classificação automática ML de propuestas de Brasil Participativo) - Residência TIC BRISA / UnB-FGA / LAPPIS</t>
+          <t>GeTAU — Gestión del Arbolado Urbano (Córdoba)</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -996,17 +996,17 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Pipeline BERTopic + LLMs sobre decenas de miles de propuestas ciudadanas reales (Plano Clima, PPA Participativo, Congresso da Juventude) en la plataforma federal Brasil Participativo; clasifica con vocabulario controlado VCGE y genera reportes.</t>
+          <t>GeTAU es una WebApp de la ciudad de Córdoba (Argentina) que combina inteligencia artificial, geolocalización y participación vecinal para el monitoreo y la gestión del arbolado urbano: la ciudadanía georreferencia, releva y monitorea ejemplares (nuevos y existentes) y cada árbol queda con una ficha de especie, ubicación, estado sanitario y necesidades de cuidado, con trazabilidad completa. Desarrollada por jóvenes de la ONG Acción Ambiental junto a la Facultad de Ciencias Exactas, Físicas y Naturales de la Universidad Nacional de Córdoba (UNC) y difundida por el laboratorio de innovación municipal CorLab. Objetivo declarado: dar al municipio y a la vecindad información precisa para planificar reforestaciones, prevenir riesgos (p. ej. caída de ejemplares) y garantizar la supervivencia de los árboles (activa a 2025, con cobertura de prensa hasta jul-2026).</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/ResidenciaTICBrisa/BP-Classificador-de-Propostas</t>
+          <t>https://corlab.cordoba.gob.ar/getau-la-app-cordobesa-para-el-cuidado-inteligente-de-arboles/ / https://cordoba.gob.ar/getau-aplicacion-arbolado-urbano/ / https://hoydia.com.ar/ambiente/getau-la-app-cordobesa-que-invita-a-vecinos-a-cuidar-y-mapear-los-arboles-de-su-barrio/ / https://g5noticias.cl/2026/07/15/arboles-en-riesgo-la-app-que-usa-ia-y-datos-de-vecinos-para-ayudar-a-prevenir-caidas/</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>NO ENTRA POR DOBLE CONTEO. Este candidato (BP-Classificador-de-Propostas, Residência TIC BRISA / UnB-FGA / LAPPIS) es el MISMO caso ya contabilizado en la ficha BR-brasil-participativo-clustering-semantic, no un caso distinto. Prueba directa: (a) esa ficha YA CITA este mismo repositorio (https://github.com/ResidenciaTICBrisa/BP-Classificador-de-Propostas) entre sus fuentes fetcheadas (Fase 2 del pipeline), y (b) el clasificador es parte del mismo pipeline de IA sobre las propuestas de Brasil Participativo (mismo corpus y mismos desarrolladores UnB/BRISA). Contarlo aparte duplicaría una iniciativa ya incluida → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/gates/fase2_estado.md (fuente GitHub fetcheada para esa ficha), ficha conciliada BR-brasil-participativo y URL del candidato]</t>
+          <t>NO ENTRA (revisión jul-2026 a pedido del equipo; la 2ª opinión coincide con el juicio del aportante). La «participación» de GeTAU es aporte de DATOS/observaciones — ciencia ciudadana y censo/mapeo colaborativo del arbolado (los vecinos georreferencian ejemplares y cargan especie, estado y cuidados) — y la IA opera sobre esos datos de árboles (identificación/estado y prevención de riesgo de caída), NO sobre el contenido de aportes de un proceso de participación ciudadana. No existe consulta pública, deliberación, presupuesto participativo, referendo ni decisión ciudadana asociada. Criterio corregido: civic tech de reporte/servicio/monitoreo que no es un proceso participativo → NO ENTRA (análogo a ParticipACT Brasil, dIAra CR, Pa' que veás CO y Satellites On Fire AR, todos excluidos). Reevaluable solo si el municipio la integrara a un proceso decisorio real (p. ej. planificación participativa del arbolado con IA sobre las propuestas ciudadanas). [Verificación: el fetch directo de corlab.cordoba.gob.ar y de la prensa fue bloqueado por el proxy del entorno; evaluación basada en la descripción aportada por el equipo y en resultados de búsqueda (Municipalidad de Córdoba «GeTAU ya está activa: una aplicación participativa que trabaja en la gestión del arbolado urbano»; hoydia.com.ar 15-oct-2025 «invita a vecinos a cuidar y mapear los árboles de su barrio»; g5noticias.cl 15-jul-2026 «la app que usa IA y datos de vecinos para ayudar a prevenir caídas»).]</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Cátedra Brasil / Co:Lab USP - IA generativa en presupuesto participativo (SP)</t>
+          <t>BP-Classificador de Propostas (indexação/classificação automática ML de propuestas de Brasil Participativo) - Residência TIC BRISA / UnB-FGA / LAPPIS</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -1028,17 +1028,17 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Investigación (Co:Lab USP, José Carlos Vaz) sobre IA generativa que ayuda a la ciudadanía a redactar y estructurar propuestas en el presupuesto participativo de São Paulo; en curso (pesquisas em andamento), no confirmado como despliegue oficial.</t>
+          <t>Pipeline BERTopic + LLMs sobre decenas de miles de propuestas ciudadanas reales (Plano Clima, PPA Participativo, Congresso da Juventude) en la plataforma federal Brasil Participativo; clasifica con vocabulario controlado VCGE y genera reportes.</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>https://colab.each.usp.br/blog/2025/03/28/a-ia-generativa-e-o-futuro-da-participacao-cidada-pesquisas-em-andamento/</t>
+          <t>https://github.com/ResidenciaTICBrisa/BP-Classificador-de-Propostas</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Investigación académica en curso ('pesquisas em andamento') sobre IA generativa para participación: sin despliegue con ciudadanos ni proceso propio (verificado). Estudio sin despliegue → NO. Decisión del equipo.</t>
+          <t>NO ENTRA POR DOBLE CONTEO. Este candidato (BP-Classificador-de-Propostas, Residência TIC BRISA / UnB-FGA / LAPPIS) es el MISMO caso ya contabilizado en la ficha BR-brasil-participativo-clustering-semantic, no un caso distinto. Prueba directa: (a) esa ficha YA CITA este mismo repositorio (https://github.com/ResidenciaTICBrisa/BP-Classificador-de-Propostas) entre sus fuentes fetcheadas (Fase 2 del pipeline), y (b) el clasificador es parte del mismo pipeline de IA sobre las propuestas de Brasil Participativo (mismo corpus y mismos desarrolladores UnB/BRISA). Contarlo aparte duplicaría una iniciativa ya incluida → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/gates/fase2_estado.md (fuente GitHub fetcheada para esa ficha), ficha conciliada BR-brasil-participativo y URL del candidato]</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Participe+ (ParticipeMais) - app estudiantil UnB-MDS de IA sobre contenidos de Brasil Participativo</t>
+          <t>Cátedra Brasil / Co:Lab USP - IA generativa en presupuesto participativo (SP)</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
@@ -1065,12 +1065,12 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/unb-mds/ParticipeMais</t>
+          <t>https://colab.each.usp.br/blog/2025/03/28/a-ia-generativa-e-o-futuro-da-participacao-cidada-pesquisas-em-andamento/</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>NO ENTRA. Aunque tecnicamente la IA SI procesa el CONTENIDO de los aportes (agrupa por temas via HDBSCAN y clasifica en eixos por similitud semantica, ademas de resumir con LLM), el candidato incumple una condicion NECESARIA del criterio de inclusion ('SI solo si caso distinto, DESPLEGADO OFICIALMENTE'): es un proyecto ESTUDIANTIL de la disciplina Métodos de Desenvolvimento de Software (UnB-MDS) construido sobre los datos públicos de Brasil Participativo, sin adopción ni despliegue oficial en la plataforma, y sobre el mismo corpus del caso ya incluido → estudio/ejercicio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: repositorio del candidato (github.com/unb-mds/ParticipeMais) y regla de elegibilidad de la pestaña Instrucciones del insumo]</t>
+          <t>Investigación académica en curso ('pesquisas em andamento') sobre IA generativa para participación: sin despliegue con ciudadanos ni proceso propio (verificado). Estudio sin despliegue → NO. Decisión del equipo.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Projeto Lumina - análise de sentimentos das propostas de Brasil Participativo (projeto estudantil UnB-MDS)</t>
+          <t>Participe+ (ParticipeMais) - app estudiantil UnB-MDS de IA sobre contenidos de Brasil Participativo</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -1092,29 +1092,29 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Pipeline BERTopic + LLMs sobre decenas de miles de propuestas ciudadanas reales (Plano Clima, PPA Participativo, Congresso da Juventude) en la plataforma federal Brasil Participativo; clasifica con vocabulario controlado VCGE y genera reportes.</t>
+          <t>Investigación (Co:Lab USP, José Carlos Vaz) sobre IA generativa que ayuda a la ciudadanía a redactar y estructurar propuestas en el presupuesto participativo de São Paulo; en curso (pesquisas em andamento), no confirmado como despliegue oficial.</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/unb-mds/2024-2-Lumina</t>
+          <t>https://github.com/unb-mds/ParticipeMais</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>NO ENTRA. Aunque la IA sí actúa sobre el CONTENIDO de aportes ciudadanos (análisis de sentimiento positivo/negativo/neutro de las propuestas y comentarios de Brasil Participativo, rol_IA=contenido), falla el requisito de DESPLIEGUE OFICIAL: Projeto Lumina es un EJERCICIO ACADÉMICO de la disciplina 'Métodos de Desenvolvimento de Software' (UnB-MDS, semestre 2024-2), sin adopción ni despliegue oficial en la plataforma → estudio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: repositorio del candidato (github.com/unb-mds/2024-2-Lumina) y regla de elegibilidad]</t>
+          <t>NO ENTRA. Aunque tecnicamente la IA SI procesa el CONTENIDO de los aportes (agrupa por temas via HDBSCAN y clasifica en eixos por similitud semantica, ademas de resumir con LLM), el candidato incumple una condicion NECESARIA del criterio de inclusion ('SI solo si caso distinto, DESPLEGADO OFICIALMENTE'): es un proyecto ESTUDIANTIL de la disciplina Métodos de Desenvolvimento de Software (UnB-MDS) construido sobre los datos públicos de Brasil Participativo, sin adopción ni despliegue oficial en la plataforma, y sobre el mismo corpus del caso ya incluido → estudio/ejercicio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: repositorio del candidato (github.com/unb-mds/ParticipeMais) y regla de elegibilidad de la pestaña Instrucciones del insumo]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Participa Pudahuel — Presupuesto Participativo deliberativo (plataforma Go Vocal/CitizenLab)</t>
+          <t>Projeto Lumina - análise de sentimentos das propostas de Brasil Participativo (projeto estudantil UnB-MDS)</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -1124,17 +1124,17 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>«Participa Pudahuel — Presupuesto Participativo deliberativo (plataforma Go Vocal/CitizenLab)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
+          <t>Pipeline BERTopic + LLMs sobre decenas de miles de propuestas ciudadanas reales (Plano Clima, PPA Participativo, Congresso da Juventude) en la plataforma federal Brasil Participativo; clasifica con vocabulario controlado VCGE y genera reportes.</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>https://participa.mpudahuel.cl/</t>
+          <t>https://github.com/unb-mds/2024-2-Lumina</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Presupuesto participativo real, pero solo se confirma que la plataforma (Go Vocal) tiene el módulo de IA/NLP de fábrica; NO hay traza de que Pudahuel lo activara sobre los aportes (usa_IA_en_proceso 'no-claro', sin evidencia). Sin uso de IA verificado → NO. Decisión del equipo.</t>
+          <t>NO ENTRA. Aunque la IA sí actúa sobre el CONTENIDO de aportes ciudadanos (análisis de sentimiento positivo/negativo/neutro de las propuestas y comentarios de Brasil Participativo, rol_IA=contenido), falla el requisito de DESPLIEGUE OFICIAL: Projeto Lumina es un EJERCICIO ACADÉMICO de la disciplina 'Métodos de Desenvolvimento de Software' (UnB-MDS, semestre 2024-2), sin adopción ni despliegue oficial en la plataforma → estudio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: repositorio del candidato (github.com/unb-mds/2024-2-Lumina) y regla de elegibilidad]</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Senador Virtual / CrowdLaw (GobLab UAI + IMFD)</t>
+          <t>Participa Pudahuel — Presupuesto Participativo deliberativo (plataforma Go Vocal/CitizenLab)</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -1156,17 +1156,17 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Investigación (GobLab UAI + IMFD, 2018-2023) sobre NLP aplicado a los aportes ciudadanos legislativos de la plataforma Senador Virtual del Senado (16 años activa); no verificado en producción.</t>
+          <t>«Participa Pudahuel — Presupuesto Participativo deliberativo (plataforma Go Vocal/CitizenLab)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>https://goblab.uai.cl/en/16-years-of-crowdlaw-in-the-chilean-parliament/</t>
+          <t>https://participa.mpudahuel.cl/</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>2a PASADA (resuelve DUDA -&gt; NO). La plataforma Senador Virtual / Congreso Virtual es un proceso participativo digital del Congreso de Chile (gobierno nacional) plenamente activo y consolidado (&gt;16 anios, &gt;130.000 participantes), pero la plataforma en si NO usa IA sobre el contenido de los aportes y el trabajo de NLP/CrowdLaw documentado (GobLab UAI + IMFD, 2018-2023) es investigación académica sobre los datos de la plataforma, sin verificación de aplicación en producción → sin IA institucional desplegada sobre los aportes → NO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/candidatos.csv (señal/nota del candidato), data/gates/gate1_decision.md y URL del caso (goblab.uai.cl)]</t>
+          <t>Presupuesto participativo real, pero solo se confirma que la plataforma (Go Vocal) tiene el módulo de IA/NLP de fábrica; NO hay traza de que Pudahuel lo activara sobre los aportes (usa_IA_en_proceso 'no-claro', sin evidencia). Sin uso de IA verificado → NO. Decisión del equipo.</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Viña Decide — Primer Presupuesto Participativo de Viña del Mar (plataforma Go Vocal/CitizenLab)</t>
+          <t>Senador Virtual / CrowdLaw (GobLab UAI + IMFD)</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -1188,29 +1188,29 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>Uso de IA para analizar datos cualitativos en consulta ciudadana.</t>
+          <t>Investigación (GobLab UAI + IMFD, 2018-2023) sobre NLP aplicado a los aportes ciudadanos legislativos de la plataforma Senador Virtual del Senado (16 años activa); no verificado en producción.</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>https://vinadecide.cl/pages/presupuestoparticipativo</t>
+          <t>https://goblab.uai.cl/en/16-years-of-crowdlaw-in-the-chilean-parliament/</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Presupuesto participativo real sobre plataforma Go Vocal, pero no se encontró en el informe ejecutivo ninguna traza de uso de IA sobre los aportes (usa_IA_en_proceso 'no-claro', sin evidencia). Sin uso de IA verificado → NO. Decisión del equipo.</t>
+          <t>2a PASADA (resuelve DUDA -&gt; NO). La plataforma Senador Virtual / Congreso Virtual es un proceso participativo digital del Congreso de Chile (gobierno nacional) plenamente activo y consolidado (&gt;16 anios, &gt;130.000 participantes), pero la plataforma en si NO usa IA sobre el contenido de los aportes y el trabajo de NLP/CrowdLaw documentado (GobLab UAI + IMFD, 2018-2023) es investigación académica sobre los datos de la plataforma, sin verificación de aplicación en producción → sin IA institucional desplegada sobre los aportes → NO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/candidatos.csv (señal/nota del candidato), data/gates/gate1_decision.md y URL del caso (goblab.uai.cl)]</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Atlántico – Plan de Ordenamiento Departamental (POD) 2025-2050 / plataforma LITA</t>
+          <t>Viña Decide — Primer Presupuesto Participativo de Viña del Mar (plataforma Go Vocal/CitizenLab)</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -1220,17 +1220,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Proceso de formulación participativa del Plan de Ordenamiento Departamental (POD) 2025-2050 del Atlántico (Colombia), convocado por la Gobernación con mesas y talleres subregionales. En paralelo, la Gobernación presenta la plataforma LITA, una base de datos con IA para almacenar, procesar y estructurar información técnica territorial y cruzar datos técnicos/geoespaciales que alimentan el diagnóstico del plan (nota de prensa de la Gobernación, 2025).</t>
+          <t>Uso de IA para analizar datos cualitativos en consulta ciudadana.</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>https://www.atlantico.gov.co/index.php/noticias/prensa-planeacion/27250-plan-de-ordenamiento-departamental-toma-forma-en-el-atlantico</t>
+          <t>https://vinadecide.cl/pages/presupuestoparticipativo</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>NO ELEGIBLE. Dentro de un proceso participativo real (POD con mesas/talleres subregionales), la IA (plataforma LITA / base de datos con IA) cumple funciones de ALMACENAMIENTO, PROCESAMIENTO y ESTRUCTURACIÓN de información técnica territorial y CRUCE de datos técnicos/geoespaciales de punta para actualizar el diagnóstico y los instrumentos del plan — es infraestructura de datos al servicio de los equipos formuladores, NO análisis del CONTENIDO de los aportes ciudadanos de las mesas y talleres → NO ELEGIBLE. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada y la nota de prensa de la Gobernación del Atlántico (URL del caso)]</t>
+          <t>Presupuesto participativo real sobre plataforma Go Vocal, pero no se encontró en el informe ejecutivo ninguna traza de uso de IA sobre los aportes (usa_IA_en_proceso 'no-claro', sin evidencia). Sin uso de IA verificado → NO. Decisión del equipo.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Citibeats + PNUD Colombia (analítica de datos para la deliberación pública juvenil)</t>
+          <t>Atlántico – Plan de Ordenamiento Departamental (POD) 2025-2050 / plataforma LITA</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -1252,17 +1252,17 @@
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>El Laboratorio de Aceleración del PNUD usó Citibeats (IA) para monitorear y agrupar en tiempo real opiniones y propuestas de deliberación pública juvenil, identificando tópicos y clasificando los inputs ciudadanos.</t>
+          <t>Proceso de formulación participativa del Plan de Ordenamiento Departamental (POD) 2025-2050 del Atlántico (Colombia), convocado por la Gobernación con mesas y talleres subregionales. En paralelo, la Gobernación presenta la plataforma LITA, una base de datos con IA para almacenar, procesar y estructurar información técnica territorial y cruzar datos técnicos/geoespaciales que alimentan el diagnóstico del plan (nota de prensa de la Gobernación, 2025).</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/colombia/blog/analitica-de-datos-para-mejorar-la-deliberacion-publica-en-colombia</t>
+          <t>https://www.atlantico.gov.co/index.php/noticias/prensa-planeacion/27250-plan-de-ordenamiento-departamental-toma-forma-en-el-atlantico</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Escucha social de redes abiertas (Twitter/Facebook) durante el paro de 2021: no hay proceso participativo convocado (verificado). Misma regla que U-Report (solo opinión) → NO. Decisión del equipo.</t>
+          <t>NO ELEGIBLE. Dentro de un proceso participativo real (POD con mesas/talleres subregionales), la IA (plataforma LITA / base de datos con IA) cumple funciones de ALMACENAMIENTO, PROCESAMIENTO y ESTRUCTURACIÓN de información técnica territorial y CRUCE de datos técnicos/geoespaciales de punta para actualizar el diagnóstico y los instrumentos del plan — es infraestructura de datos al servicio de los equipos formuladores, NO análisis del CONTENIDO de los aportes ciudadanos de las mesas y talleres → NO ELEGIBLE. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada y la nota de prensa de la Gobernación del Atlántico (URL del caso)]</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
+          <t>Citibeats + PNUD Colombia (analítica de datos para la deliberación pública juvenil)</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
@@ -1284,17 +1284,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>51 diálogos regionales, 250.000 participantes, 89.788 propuestas ciudadanas; una 'Unidad de Científicos de Datos' del DNP las sistematizó (análisis por frecuencia/recurrencia).</t>
+          <t>El Laboratorio de Aceleración del PNUD usó Citibeats (IA) para monitorear y agrupar en tiempo real opiniones y propuestas de deliberación pública juvenil, identificando tópicos y clasificando los inputs ciudadanos.</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>https://dialogosregionales.dnp.gov.co/</t>
+          <t>https://www.undp.org/es/colombia/blog/analitica-de-datos-para-mejorar-la-deliberacion-publica-en-colombia</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Participación real, pero el análisis fue manual/cualitativo; solo text-analytics ligero (nubes de palabras + tabulación), sin NLP sobre el contenido (verificado). Decisión del equipo.</t>
+          <t>Escucha social de redes abiertas (Twitter/Facebook) durante el paro de 2021: no hay proceso participativo convocado (verificado). Misma regla que U-Report (solo opinión) → NO. Decisión del equipo.</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>IA para participación en el POT de Bogotá (Control Visible / Auditoría General)</t>
+          <t>DNP - Diálogos Regionales Vinculantes (PND 2022-2026)</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -1316,17 +1316,17 @@
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>Artículo (Revista de la Auditoría General, jun-2025) que aplica modelos de IA al contenido de aportes ciudadanos en la planificación urbana (POT) de Bogotá; metodología mixta con 395 ciudadanos.</t>
+          <t>51 diálogos regionales, 250.000 participantes, 89.788 propuestas ciudadanas; una 'Unidad de Científicos de Datos' del DNP las sistematizó (análisis por frecuencia/recurrencia).</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>https://controlvisible.auditoria.gov.co/index.php/rcf/article/view/63</t>
+          <t>https://dialogosregionales.dnp.gov.co/</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>NO ENTRA. El criterio de elegibilidad exige que dentro de un proceso participativo se DESPLIEGUE IA real (institucional) sobre el CONTENIDO de los aportes ciudadanos. El caso documentado es un ARTÍCULO ACADÉMICO (Fundación Universitaria del Área Andina, Maestría en Innovación; publicado en la revista de Control Visible de la Auditoría General de la República, jun-2025) que aplica modelos de IA al contenido de aportes ciudadanos del POT (metodología mixta, 395 participantes) como propuesta/piloto de investigación, sin despliegue institucional en el proceso participativo → estudio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/candidatos.csv (señal del candidato CO-ia-para-participacion-en-el-pot-de-bogot) y URL del caso (controlvisible.auditoria.gov.co)]</t>
+          <t>Participación real, pero el análisis fue manual/cualitativo; solo text-analytics ligero (nubes de palabras + tabulación), sin NLP sobre el contenido (verificado). Decisión del equipo.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>ISIDataInsights / Reto de Ciudad 'Datos con Historia' (SDP Bogotá)</t>
+          <t>IA para participación en el POT de Bogotá (Control Visible / Auditoría General)</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Herramienta de IA ganadora del concurso abierto SDP Bogotá + Maloka (oct-nov 2024) que procesa documentos e identifica patrones clave en los aportes ciudadanos y documentos de planificación distrital; en implementación para integrarse a la Secretaría Distrital de Planeación (Plan de Desarrollo 2024-2028).</t>
+          <t>Artículo (Revista de la Auditoría General, jun-2025) que aplica modelos de IA al contenido de aportes ciudadanos en la planificación urbana (POT) de Bogotá; metodología mixta con 395 ciudadanos.</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>https://www.sdp.gov.co/noticias/bogota-cuenta-herramienta-innovadora-abordar-los-problemas-urbanos-aporte-de-la-ciudadania</t>
+          <t>https://controlvisible.auditoria.gov.co/index.php/rcf/article/view/63</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>EXCLUIDO (reafirmado en reexamen jul-2026). Herramienta ganadora del reto de innovación abierta «Datos con Historia» de la Secretaría Distrital de Planeación (SDP), desarrollada por la empresa IGG (dic-2024). Alcanzó solo un «producto mínimo viable funcional, probado en el contexto institucional»; su integración a los sistemas del Distrito y su aplicación sobre los aportes ciudadanos están en tiempo FUTURO («será integrada», «se incorporará», «inicia la tercera etapa, en la cual se implementará»). Sin evidencia (2024-2026) de despliegue real sobre un proceso participativo concreto → cae en la exclusión (e): herramienta de reto/desafío sin despliegue. RELACIÓN CON CHATICO (verificada): son herramientas INDEPENDIENTES — distinta entidad (SDP vs Secretaría General / Consejería Distrital de TIC), distinto desarrollador y distinta función (ISIDataInsights «procesaría» documentos de planeación; Chatico recolecta y clasifica aportes). NO hay solapamiento de corpus ni doble conteo: el único proceso participativo real con aportes ciudadanos (Plan Distrital de Desarrollo «Bogotá Camina Segura», 147.422 aportes) lo ejecutó Chatico —ya contado— y las notas oficiales del Plan NO mencionan a ISIDataInsights, por lo que no puede «heredar» ese despliegue para calificar. Chatico permanece bien atribuido.</t>
+          <t>NO ENTRA. El criterio de elegibilidad exige que dentro de un proceso participativo se DESPLIEGUE IA real (institucional) sobre el CONTENIDO de los aportes ciudadanos. El caso documentado es un ARTÍCULO ACADÉMICO (Fundación Universitaria del Área Andina, Maestría en Innovación; publicado en la revista de Control Visible de la Auditoría General de la República, jun-2025) que aplica modelos de IA al contenido de aportes ciudadanos del POT (metodología mixta, 395 participantes) como propuesta/piloto de investigación, sin despliegue institucional en el proceso participativo → estudio sin despliegue → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/candidatos.csv (señal del candidato CO-ia-para-participacion-en-el-pot-de-bogot) y URL del caso (controlvisible.auditoria.gov.co)]</t>
         </is>
       </c>
     </row>
@@ -1370,20 +1370,52 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
+          <t>ISIDataInsights / Reto de Ciudad 'Datos con Historia' (SDP Bogotá)</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Herramienta de IA ganadora del concurso abierto SDP Bogotá + Maloka (oct-nov 2024) que procesa documentos e identifica patrones clave en los aportes ciudadanos y documentos de planificación distrital; en implementación para integrarse a la Secretaría Distrital de Planeación (Plan de Desarrollo 2024-2028).</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sdp.gov.co/noticias/bogota-cuenta-herramienta-innovadora-abordar-los-problemas-urbanos-aporte-de-la-ciudadania</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>EXCLUIDO (reafirmado en reexamen jul-2026). Herramienta ganadora del reto de innovación abierta «Datos con Historia» de la Secretaría Distrital de Planeación (SDP), desarrollada por la empresa IGG (dic-2024). Alcanzó solo un «producto mínimo viable funcional, probado en el contexto institucional»; su integración a los sistemas del Distrito y su aplicación sobre los aportes ciudadanos están en tiempo FUTURO («será integrada», «se incorporará», «inicia la tercera etapa, en la cual se implementará»). Sin evidencia (2024-2026) de despliegue real sobre un proceso participativo concreto → cae en la exclusión (e): herramienta de reto/desafío sin despliegue. RELACIÓN CON CHATICO (verificada): son herramientas INDEPENDIENTES — distinta entidad (SDP vs Secretaría General / Consejería Distrital de TIC), distinto desarrollador y distinta función (ISIDataInsights «procesaría» documentos de planeación; Chatico recolecta y clasifica aportes). NO hay solapamiento de corpus ni doble conteo: el único proceso participativo real con aportes ciudadanos (Plan Distrital de Desarrollo «Bogotá Camina Segura», 147.422 aportes) lo ejecutó Chatico —ya contado— y las notas oficiales del Plan NO mencionan a ISIDataInsights, por lo que no puede «heredar» ese despliegue para calificar. Chatico permanece bien atribuido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
           <t>GaitanIA</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>«GaitanIA». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E31" s="9" t="inlineStr">
         <is>
           <t>https://gaitanaia.org/
  https://www.lasillavacia.com/en-vivo/gaitana-ia-la-herramienta-de-un-resguardo-indigena-para-llegar-al-congreso/
@@ -1394,53 +1426,21 @@
  https://thebogotapost.com/gaitana-ia-the-ai-candidate-that-ran-in-colombias-elections/55921/</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>(1) Cerosetenta/070 (Uniandes, 07-mar-2026): «Gaitana no es una candidata. Se trata más bien de un mecanismo de campaña electoral» para las listas de C. Redondo (Senado) y A. Rincón (Cámara), circunscripción indígena. (2) El mecanismo participativo insignia (curul híbrida: votos legislativos definidos por consulta digital a la comunidad) era CONDICIONAL a ganar; obtuvieron &lt;3.000 votos el 8-mar-2026 (se requerían ~25.000) y no ganaron curul → nunca operó (anuncio sin implementación). (3) La votación digital de presupuestos del cabildo Zenú (sustento del coding «Presupuestos Participativos») no tiene verificación independiente: el propio Redondo describió el origen a Rest of World como «a simple website to make it easier for people to ask questions, and get information». (4) Rol de la IA no verificable: Sáenz (Karisma): «little clarity on how consensus is reached, how it will be governed, and what AI's role is»; el chatbot alucina trabajo con comunidades (rep. del pueblo Nasa lo desmiente; Redondo: «si la IA dice esto, es porque está pasando»). (5) Jul-2026: gaitanaia.org reconvertido en proyecto-manifiesto («manual civilizatorio», Repúblicas Digitales Participativas) con contenido tras login; sin proceso participativo público operando. VERIFICADO que SÍ usa IA: chatbot LLM (DeepSeek adaptado a cosmovisión Zenú) + avatar/contenidos de campaña generados con IA + foro de campaña donde la IA «mediaría» (solo dicho por creadores, mecánica opaca). NO-IA: votación y trazabilidad = blockchain/smart contracts. Si el equipo decide mantenerlo pese a todo: bajar Confianza a BAJA, quitar «Presupuestos Participativos», Nivel 1.0 y rol_IA sin confirmar. Impacto de excluir: CO pasa de 4 a 3 iniciativas (banda Cantidad 50→25); CO conserva Presupuestos Participativos vía Chatico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>GT</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>«Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>https://portal.segeplan.gob.gt/segeplan/?p=14176</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>El criterio ELEGIBLE exige que la IA generativa se use para SISTEMATIZAR/CLASIFICAR/RESUMIR el CONTENIDO de los aportes de los diagnosticos participativos (Consejos de Desarrollo COCODES/COMUDES) en los Planes de Desarrollo Municipal (PDM). Toda la evidencia primaria y secundaria (nota SEGEPLAN ?p=14176 y cobertura relacionada) describe la plataforma de modelos generativos como apoyo interno a la formulación/actualización de instrumentos de planificación por equipos técnicos, sin evidencia de IA aplicada al contenido de los aportes participativos → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: URL del caso (portal.segeplan.gob.gt/segeplan/?p=14176) y data/gates/descubrimiento_paises_flacos.md («ENIA/SEGEPLAN = uso interno o consulta sobre IA»)]</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>GT</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
+          <t>Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -1450,29 +1450,29 @@
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>Gobierno estatal recolectó opiniones de 26.000+ ciudadanos en talleres en 46 municipios; IA analiza los aportes para identificar patrones de los principales problemas que alimentan los ejes del plan de gobierno (lanzado feb-2025).</t>
+          <t>«Plataforma de modelos generativos de IA de SEGEPLAN + Red Ciudadana (Guatemala)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>https://armemosunplan.mx/propuestas-ciudadanas/</t>
+          <t>https://portal.segeplan.gob.gt/segeplan/?p=14176</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Proceso participativo real y masivo (675.484 participaciones; 15.899 propuestas), pero NO hay evidencia de uso de IA para analizar/agrupar/clasificar el contenido de las propuestas (usa_IA_en_proceso 'no'). Sin uso de IA → NO. Decisión del equipo.</t>
+          <t>El criterio ELEGIBLE exige que la IA generativa se use para SISTEMATIZAR/CLASIFICAR/RESUMIR el CONTENIDO de los aportes de los diagnosticos participativos (Consejos de Desarrollo COCODES/COMUDES) en los Planes de Desarrollo Municipal (PDM). Toda la evidencia primaria y secundaria (nota SEGEPLAN ?p=14176 y cobertura relacionada) describe la plataforma de modelos generativos como apoyo interno a la formulación/actualización de instrumentos de planificación por equipos técnicos, sin evidencia de IA aplicada al contenido de los aportes participativos → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: URL del caso (portal.segeplan.gob.gt/segeplan/?p=14176) y data/gates/descubrimiento_paises_flacos.md («ENIA/SEGEPLAN = uso interno o consulta sobre IA»)]</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>PY</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)</t>
+          <t>Jalisco - Consulta ¡Armemos un Plan! (Plan Estatal de Desarrollo y Gobernanza 2024-2030)</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -1482,115 +1482,115 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>«Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
+          <t>Gobierno estatal recolectó opiniones de 26.000+ ciudadanos en talleres en 46 municipios; IA analiza los aportes para identificar patrones de los principales problemas que alimentan los ejes del plan de gobierno (lanzado feb-2025).</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/paraguay/blog/consultas-ciudadanas-sobre-ia-en-paraguay-visiones-diversas-entre-el-campo-y-la-ciudad</t>
+          <t>https://armemosunplan.mx/propuestas-ciudadanas/</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>El criterio ELEGIBLE exige que dentro de un proceso participativo convocado se use IA (NLP/ML/clustering/sentimiento) SOBRE EL CONTENIDO de los aportes. Aquí ocurre lo contrario: (1) la IA es el TEMA de la consulta (se pregunta a la ciudadania por su percepcion de la IA), y (2) el ANÁLISIS de los aportes de las consultas fue realizado por el equipo (AccLab PNUD + Columbia SIPA + MITIC) con métodos convencionales, sin traza de NLP/ML sobre el contenido → la IA es el tema, no la herramienta → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada (puntos 1-2) y el blog del PNUD Paraguay (URL del caso)]</t>
+          <t>Proceso participativo real y masivo (675.484 participaciones; 15.899 propuestas), pero NO hay evidencia de uso de IA para analizar/agrupar/clasificar el contenido de las propuestas (usa_IA_en_proceso 'no'). Sin uso de IA → NO. Decisión del equipo.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
+          <t>PY</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>«Consultas ciudadanas sobre IA en Paraguay - PNUD Accelerator Lab (AccLab) + Columbia SIPA + MITIC / insumo del diagnóstico AILA (Atlas de IA)». Caso identificado en el descubrimiento 2026 y no incluido; la descripción técnica y la razón de no inclusión se detallan en la columna «Motivo y detalles de la exclusión».</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>https://www.undp.org/es/paraguay/blog/consultas-ciudadanas-sobre-ia-en-paraguay-visiones-diversas-entre-el-campo-y-la-ciudad</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>El criterio ELEGIBLE exige que dentro de un proceso participativo convocado se use IA (NLP/ML/clustering/sentimiento) SOBRE EL CONTENIDO de los aportes. Aquí ocurre lo contrario: (1) la IA es el TEMA de la consulta (se pregunta a la ciudadania por su percepcion de la IA), y (2) el ANÁLISIS de los aportes de las consultas fue realizado por el equipo (AccLab PNUD + Columbia SIPA + MITIC) con métodos convencionales, sin traza de NLP/ML sobre el contenido → la IA es el tema, no la herramienta → NO ENTRA. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada (puntos 1-2) y el blog del PNUD Paraguay (URL del caso)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>TT</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>engage.gov.tt corre sobre Go Vocal (confirmado por URL interna 'e-democracy-govocal-internal'), lanzada feb-2025 para el NDTS 2024-2027 (planificación nacional participativa). Go Vocal incorpora NLP de sensemaking, pero NO está confirmado que la instancia TT lo active; AskNDTS es chatbot FAQ (excluido). Evidencia (validación): Go Vocal Support Base (AI Analysis): 'Access to this feature depends on your plan. Advanced Sensemaking with auto-insights is available in the Premium plan.' -&gt; la IA/NLP de Go Vocal NO es automatica, depende del plan; y para EngageTT solo se documenta 'feedback via surveys and polls'/Open Forum/ideas, SIN mencion de analisis automatico por IA de los aportes. No se halla evidencia de activacion del NLP sobre el contenido en la instancia TT. 3a PASADA (refuerzo): Oxford Insights, 'The country's AI utilisation for citizens is concentrated in a robust Chatbot programme' (mas 'deployment of large language models for internal development purposes') -&gt; la IA ciudadana de TT es el chatbot, NO el analisis de aportes.</t>
         </is>
       </c>
-      <c r="E34" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>https://engage.gov.tt/ideas/ndts-2025-actionable-feedback-implementation-plan
 https://www.govocal.com/plans
 https://support.govocal.com/en/articles/9015305-faq-on-our-ai-sensemaking-tool</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>EngageTT aloja MÚLTIPLES proyectos → plan Essential (1 proyecto activo) improbable → el módulo IA probablemente está DISPONIBLE en el back-office de la instancia TT. PERO disponible ≠ usado: (1) son funciones admin-side invisibles desde afuera y la moderación NLP es un toggle opcional de settings; (2) tras 4 pasadas no hay evidencia pública de USO (ni resúmenes IA ni moderación IA) sobre los aportes del NDTS; (3) la única IA ciudadana confirmada sigue siendo chatbots informativos (AskNDTS; Anansi en ttconnect = «AI-powered national digital assistant» para servicios, con booking y derivación a agente humano) = atención ciudadana, no logística del proceso; (4) RAM-UNESCO usa IA solo como tema</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>UY</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
-        </is>
-      </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Consulta pública y proceso de participación multiactor «Niñas, niños, adolescentes, entornos digitales e inteligencia artificial», lanzado por el Ministerio de Educación y Cultura de Uruguay (2026). La consulta permanece abierta hasta el 10/09/2026; la fase de sistematización, análisis y validación (Fase 3) está prevista entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026.</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026. A la fecha de evaluación (2026-07-01) la fase de análisis NO se ha ejecutado, por lo que no existe aún uso de IA verificable sobre los aportes dentro de la ventana del ciclo 2026 → NO; reevaluar en el ciclo siguiente, cuando la sistematización esté ejecutada. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada (fechas del proceso) y la noticia del MEC (URL del caso)]</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>UY</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>Boti</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>Base 2025 — ya estaba EXCLUIDO, exclusión reconfirmada</t>
+          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>Nuevo 2026 — identificado en descubrimiento, no incluido</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Chatbot oficial de la Ciudad Autónoma de Buenos Aires, diseñado para acercar información y trámites municipales a los vecinos mediante WhatsApp y otros canales digitales Buenos Aires. Su objetivo inicial fue ofrecer respuestas precisas en ámbitos específicos antes de expandirse a múltiples temas de la ciudad. A lo largo de su operación, ha evolucionado incorporando tecnologías de inteligencia artificial generativa y módulos especializados para atender desde consultas turísticas hasta denuncias por violencia laboral (Año: 2019-25).</t>
+          <t>Consulta pública y proceso de participación multiactor «Niñas, niños, adolescentes, entornos digitales e inteligencia artificial», lanzado por el Ministerio de Educación y Cultura de Uruguay (2026). La consulta permanece abierta hasta el 10/09/2026; la fase de sistematización, análisis y validación (Fase 3) está prevista entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026.</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>https://buenosaires.gob.ar/innovacionytransformaciondigital/boti#:~:text=%C2%BFC%C3%B3mo%20puedo%20chatear%20con%20Boti,la%20Ciudad%20de%20Buenos%20Aires.</t>
+          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el 30/11/2026. A la fecha de evaluación (2026-07-01) la fase de análisis NO se ha ejecutado, por lo que no existe aún uso de IA verificable sobre los aportes dentro de la ventana del ciclo 2026 → NO; reevaluar en el ciclo siguiente, cuando la sistematización esté ejecutada. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: la propia justificación truncada (fechas del proceso) y la noticia del MEC (URL del caso)]</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>Chequeabot</t>
+          <t>Boti</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
@@ -1612,17 +1612,17 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Herramienta que detecta noticias falsas mediante el análisis automático de afirmaciones públicas (Año: 2016).</t>
+          <t>Chatbot oficial de la Ciudad Autónoma de Buenos Aires, diseñado para acercar información y trámites municipales a los vecinos mediante WhatsApp y otros canales digitales Buenos Aires. Su objetivo inicial fue ofrecer respuestas precisas en ámbitos específicos antes de expandirse a múltiples temas de la ciudad. A lo largo de su operación, ha evolucionado incorporando tecnologías de inteligencia artificial generativa y módulos especializados para atender desde consultas turísticas hasta denuncias por violencia laboral (Año: 2019-25).</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>https://chequeado.com/chequeabot/</t>
+          <t>https://buenosaires.gob.ar/innovacionytransformaciondigital/boti#:~:text=%C2%BFC%C3%B3mo%20puedo%20chatear%20con%20Boti,la%20Ciudad%20de%20Buenos%20Aires.</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>DemocracyOS</t>
+          <t>Chequeabot</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>DemocraciaOS es una plataforma digital de código abierto desarrollada por la organización argentina Democracia en Red, que busca facilitar y fortalecer la participación ciudadana en procesos democráticos (Año: 2012).</t>
+          <t>Herramienta que detecta noticias falsas mediante el análisis automático de afirmaciones públicas (Año: 2016).</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>https://www.democraciaos.org/</t>
+          <t>https://chequeado.com/chequeabot/</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>No se identifica uso de IA</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>Mapa de Oportunidades Comerciales</t>
+          <t>DemocracyOS</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
@@ -1676,17 +1676,17 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Algoritmo que cruza datos demográficos, inmobiliarios y POS para recomendar zonas de inversión a pymes (Año: 2022-25).</t>
+          <t>DemocraciaOS es una plataforma digital de código abierto desarrollada por la organización argentina Democracia en Red, que busca facilitar y fortalecer la participación ciudadana en procesos democráticos (Año: 2012).</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>https://buenosaires.gob.ar/herramientas-para-elegir-tu-futuro-local/mapa-de-oportunidades-comerciales-moc</t>
+          <t>https://www.democraciaos.org/</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>No entra en la descripción de lo que es Participación ciudadana. Se considera Civic Tech, pero no participación ciudadana</t>
+          <t>No se identifica uso de IA</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>Satellites On Fire</t>
+          <t>Mapa de Oportunidades Comerciales</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
@@ -1708,29 +1708,29 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Ciudadanos reportan focos de incendio mediante una aplicación, y la IA de visión satelital ValMapX valida y envía alertas a las autoridades provinciales (Año: 2023).</t>
+          <t>Algoritmo que cruza datos demográficos, inmobiliarios y POS para recomendar zonas de inversión a pymes (Año: 2022-25).</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>https://agencia.unq.edu.ar/?p=10126</t>
+          <t>https://buenosaires.gob.ar/herramientas-para-elegir-tu-futuro-local/mapa-de-oportunidades-comerciales-moc</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>No entra en la descripción de lo que es Participación ciudadana. Se considera Civic Tech, pero no participación ciudadana. Tampoco utiliza IA</t>
+          <t>No entra en la descripción de lo que es Participación ciudadana. Se considera Civic Tech, pero no participación ciudadana</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>Busca por voz</t>
+          <t>Satellites On Fire</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
@@ -1740,17 +1740,17 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>El Gobierno de Brasil ha lanzado una nueva funcionalidad de búsqueda por voz en el portal GOV.BR, permitiendo a los usuarios acceder a más de 4.300 servicios digitales mediante comandos de voz. Esta iniciativa, busca facilitar la ciudadanía digital, especialmente para personas con discapacidad visual o dificultades para escribir (Año: 2024-25).</t>
+          <t>Ciudadanos reportan focos de incendio mediante una aplicación, y la IA de visión satelital ValMapX valida y envía alertas a las autoridades provinciales (Año: 2023).</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.br/governodigital/pt-br/noticias/gestao-divulga-201cbusca-por-voz201d-no-gov-br-para-ampliar-inclusao-digital</t>
+          <t>https://agencia.unq.edu.ar/?p=10126</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>No entra en la descripción de lo que es Participación ciudadana. Se considera Civic Tech, pero no participación ciudadana. Tampoco utiliza IA</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>De ciudadano a senador: la inteligencia artificial y la reinvención de la elaboración legislativa en Brasil”</t>
+          <t>Busca por voz</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
@@ -1772,17 +1772,17 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>Iniciativa del Senado Federal de Brasil que busca potenciar la participación ciudadana en el proceso legislativo mediante el uso de inteligencia artificial. El propósito principal es transformar a los ciudadanos de votantes ocasionales en participantes activos en la creación de leyes, utilizando herramientas digitales y IA para facilitar y enriquecer su involucramiento en el proceso legislativo (Año: 2023).</t>
+          <t>El Gobierno de Brasil ha lanzado una nueva funcionalidad de búsqueda por voz en el portal GOV.BR, permitiendo a los usuarios acceder a más de 4.300 servicios digitales mediante comandos de voz. Esta iniciativa, busca facilitar la ciudadanía digital, especialmente para personas con discapacidad visual o dificultades para escribir (Año: 2024-25).</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>https://rebootdemocracy.ai/blog/ai-lawmaking-brazil-senate</t>
+          <t>https://www.gov.br/governodigital/pt-br/noticias/gestao-divulga-201cbusca-por-voz201d-no-gov-br-para-ampliar-inclusao-digital</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Propuesta, pero no hay datos sobre que se vaya a ejecutar</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>Fala.BR</t>
+          <t>De ciudadano a senador: la inteligencia artificial y la reinvención de la elaboración legislativa en Brasil”</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
@@ -1804,17 +1804,17 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Plataforma para solicitudes de acceso a información y manifestaciones de ouvidoria u "oficina de atención ciudadana" (reclamos, denuncias, sugerencias) (Año: 2019-25).</t>
+          <t>Iniciativa del Senado Federal de Brasil que busca potenciar la participación ciudadana en el proceso legislativo mediante el uso de inteligencia artificial. El propósito principal es transformar a los ciudadanos de votantes ocasionales en participantes activos en la creación de leyes, utilizando herramientas digitales y IA para facilitar y enriquecer su involucramiento en el proceso legislativo (Año: 2023).</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>https://falabr.cgu.gov.br/</t>
+          <t>https://rebootdemocracy.ai/blog/ai-lawmaking-brazil-senate</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>Propuesta, pero no hay datos sobre que se vaya a ejecutar</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Jaque</t>
+          <t>Fala.BR</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Secretario virtual basado en IA que guía a los ciudadanos a través de la Guía de Servicios digital del estado (portal unificado de trámites). Extrae información vía API de un catálogo centralizado y responde consultas ciudadanas sobre requisitos, horarios, ubicaciones y pasos para acceder a servicios públicosoecd.orgoecd.org. Objetivo: mejorar la experiencia ciudadana en trámites, ofreciendo atención 24/7 y estandarizada (Año: 2020–25).</t>
+          <t>Plataforma para solicitudes de acceso a información y manifestaciones de ouvidoria u "oficina de atención ciudadana" (reclamos, denuncias, sugerencias) (Año: 2019-25).</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://falabr.cgu.gov.br/</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>Mudamos</t>
+          <t>Jaque</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
@@ -1868,17 +1868,17 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Es una plataforma digital desarrollada por el Instituto de Tecnología y Sociedad de Río (ITS Rio) para facilitar la creación y firma de proyectos de ley de iniciativa popular mediante el uso de tecnología blockchain, que garantiza la seguridad y verificabilidad de las firmas digitales (Año: 2019).</t>
+          <t>Secretario virtual basado en IA que guía a los ciudadanos a través de la Guía de Servicios digital del estado (portal unificado de trámites). Extrae información vía API de un catálogo centralizado y responde consultas ciudadanas sobre requisitos, horarios, ubicaciones y pasos para acceder a servicios públicosoecd.orgoecd.org. Objetivo: mejorar la experiencia ciudadana en trámites, ofreciendo atención 24/7 y estandarizada (Año: 2020–25).</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>https://www.mudamos.org/</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>No se identifica uso de IA</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>Participa+ Brasil</t>
+          <t>Mudamos</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
@@ -1900,12 +1900,12 @@
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Participa + Brasil es una plataforma oficial del Gobierno Federal de Brasil que centraliza oportunidades de participación social, como consultas públicas, audiencias y consejos, permitiendo a los ciudadanos contribuir en la formulación de políticas públicas (Año: 2023).</t>
+          <t>Es una plataforma digital desarrollada por el Instituto de Tecnología y Sociedad de Río (ITS Rio) para facilitar la creación y firma de proyectos de ley de iniciativa popular mediante el uso de tecnología blockchain, que garantiza la seguridad y verificabilidad de las firmas digitales (Año: 2019).</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>https://www.gov.br/participamaisbrasil/pagina-inicial</t>
+          <t>https://www.mudamos.org/</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>Querido Diário</t>
+          <t>Participa+ Brasil</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
@@ -1932,17 +1932,17 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>Querido Diário es una plataforma de Open Knowledge Brasil que emplea inteligencia artificial para clasificar, contextualizar y expandir la información de los diarios oficiales municipales, haciéndolos accesibles en formato abierto y amigable. Al centralizar más de 850.000 diarios de 522 municipios, facilita el monitoreo ciudadano de actos oficiales y promueve el control social mediante búsquedas semánticas y una API abierta que integra estos datos en otras herramientas cívicas (Año: 2021-25).</t>
+          <t>Participa + Brasil es una plataforma oficial del Gobierno Federal de Brasil que centraliza oportunidades de participación social, como consultas públicas, audiencias y consejos, permitiendo a los ciudadanos contribuir en la formulación de políticas públicas (Año: 2023).</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>https://ok.org.br/projetos/querido-diario/</t>
+          <t>https://www.gov.br/participamaisbrasil/pagina-inicial</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>No se identifica uso de IA</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>Robô ALICE (CGU)</t>
+          <t>Querido Diário</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>Robô ALICE es una herramienta de inteligencia artificial desarrollada por la CGU para automatizar el análisis de datos en procesos de compras públicas, permitiendo identificar patrones y posibles irregularidades en la administración pública (Año: 2019).</t>
+          <t>Querido Diário es una plataforma de Open Knowledge Brasil que emplea inteligencia artificial para clasificar, contextualizar y expandir la información de los diarios oficiales municipales, haciéndolos accesibles en formato abierto y amigable. Al centralizar más de 850.000 diarios de 522 municipios, facilita el monitoreo ciudadano de actos oficiales y promueve el control social mediante búsquedas semánticas y una API abierta que integra estos datos en otras herramientas cívicas (Año: 2021-25).</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>https://oecd-opsi.org/innovations/robot-alice-bid-contract-and-notice-analyser/</t>
+          <t>https://ok.org.br/projetos/querido-diario/</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>Serenata.ai</t>
+          <t>Robô ALICE (CGU)</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
@@ -1996,17 +1996,17 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Serenata.ai es el sitio web oficial de la Operación Serenata de Amor, un proyecto brasileño de innovación cívica. Su objetivo principal es fiscalizar el uso de fondos públicos por parte de diputados y senadores, utilizando técnicas de IA para detectar posibles irregularidades en los reembolsos solicitados por los parlamentarios (Año: 2016-25).</t>
+          <t>Robô ALICE es una herramienta de inteligencia artificial desarrollada por la CGU para automatizar el análisis de datos en procesos de compras públicas, permitiendo identificar patrones y posibles irregularidades en la administración pública (Año: 2019).</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>https://serenata.ai/</t>
+          <t>https://oecd-opsi.org/innovations/robot-alice-bid-contract-and-notice-analyser/</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>No es participación Ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>Tira-Dúvidas TSE</t>
+          <t>Serenata.ai</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
@@ -2028,29 +2028,29 @@
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Chatbot WhatsApp con verificador automático de desinformación y búsqueda semántica de normas (Año: 2022-25).</t>
+          <t>Serenata.ai es el sitio web oficial de la Operación Serenata de Amor, un proyecto brasileño de innovación cívica. Su objetivo principal es fiscalizar el uso de fondos públicos por parte de diputados y senadores, utilizando técnicas de IA para detectar posibles irregularidades en los reembolsos solicitados por los parlamentarios (Año: 2016-25).</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>https://www.tse.jus.br/comunicacao/noticias/2022/Setembro/tira-duvidas-do-tse-no-whatsapp-ganha-ferramenta-inedita-de-checagem-de-fatos-para-as-eleicoes-2022-402542</t>
+          <t>https://serenata.ai/</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación Ciudadana</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>Caminar</t>
+          <t>Tira-Dúvidas TSE</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
@@ -2060,17 +2060,17 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>El Proyecto CAMINAR (Cámara Inteligencia Artificial) es una iniciativa de la Cámara de Diputadas y Diputados de Chile que busca modernizar el trabajo parlamentario mediante el uso de inteligencia artificial. El proyecto tiene como objetivo mejorar la eficiencia, transparencia y accesibilidad de los procesos legislativos (Año: 2023).</t>
+          <t>Chatbot WhatsApp con verificador automático de desinformación y búsqueda semántica de normas (Año: 2022-25).</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>https://parlamericas.org/uploads/documents/Presentation-OPNStaffMeeting-ProyectoCAMINARChile_MiguelLanderos-sp.pdf</t>
+          <t>https://www.tse.jus.br/comunicacao/noticias/2022/Setembro/tira-duvidas-do-tse-no-whatsapp-ganha-ferramenta-inedita-de-checagem-de-fatos-para-as-eleicoes-2022-402542</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>De acuerdo a la descripción, solo permitiría a los ciudadanos consultar</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>Modelo de inferencia de posturas en Twitter (referéndum)</t>
+          <t>Caminar</t>
         </is>
       </c>
       <c r="C52" s="12" t="inlineStr">
@@ -2092,17 +2092,17 @@
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Investigación que desarrolló un modelo de inteligencia artificial para inferir automáticamente las posturas políticas de los usuarios de Twitter durante los procesos constitucionales de 2020 y 2022. Este modelo, basado en redes neuronales convolucionales sobre grafos (Graph Convolutional Networks), analiza tanto el contenido textual de los tuits como las conexiones entre usuarios y temas para predecir si un usuario apoya o rechaza una propuesta constitucional (Año: 2023-24).</t>
+          <t>El Proyecto CAMINAR (Cámara Inteligencia Artificial) es una iniciativa de la Cámara de Diputadas y Diputados de Chile que busca modernizar el trabajo parlamentario mediante el uso de inteligencia artificial. El proyecto tiene como objetivo mejorar la eficiencia, transparencia y accesibilidad de los procesos legislativos (Año: 2023).</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2303.15532</t>
+          <t>https://parlamericas.org/uploads/documents/Presentation-OPNStaffMeeting-ProyectoCAMINARChile_MiguelLanderos-sp.pdf</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Es un estudio</t>
+          <t>De acuerdo a la descripción, solo permitiría a los ciudadanos consultar</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
+          <t>Modelo de inferencia de posturas en Twitter (referéndum)</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
@@ -2124,29 +2124,29 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>La Plataforma UCampus fue la herramienta digital oficial utilizada en el proceso constituyente de Chile en 2023, desarrollada por el Centro Tecnológico UCampus de la Facultad de Ciencias Físicas y Matemáticas de la Universidad de Chile. Su objetivo principal fue facilitar la participación ciudadana en la redacción de una nueva Constitución, ofreciendo un espacio accesible y seguro para que la ciudadanía pudiera involucrarse activamente en este proceso histórico (Año: 2023-24).</t>
+          <t>Investigación que desarrolló un modelo de inteligencia artificial para inferir automáticamente las posturas políticas de los usuarios de Twitter durante los procesos constitucionales de 2020 y 2022. Este modelo, basado en redes neuronales convolucionales sobre grafos (Graph Convolutional Networks), analiza tanto el contenido textual de los tuits como las conexiones entre usuarios y temas para predecir si un usuario apoya o rechaza una propuesta constitucional (Año: 2023-24).</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>https://ucampus.cl/ucampus-es-la-plataforma-digital-del-proceso-constitucional-2023/</t>
+          <t>https://arxiv.org/abs/2303.15532</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>Motivo 2025: «No evidencia de uso de IA» · Reconfirmación 2026: MANTENER EXCLUIDO. Existe un proceso participativo ELEGIBLE (Proceso Constitucional 2023, mecanismos de participación ciudadana con ~280 mil personas, convocado por el Estado de Chile), y UCampus (Universidad de Chile) fue el operador técnico de dos de los cuatro mecanismos (Audiencias Públicas e Iniciativa Popular de Norma), pero no se encontró evidencia de que se aplicara IA/NLP sobre el CONTENIDO de los aportes en esos mecanismos → el motivo 2025 («No evidencia de uso de IA») sigue vigente → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv (por qué se revisó) y URL del caso (ucampus.cl)]</t>
+          <t>Es un estudio</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>CO</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
+          <t>Plataforma UCampus - participación 2023 (proceso constitucional)</t>
         </is>
       </c>
       <c r="C54" s="12" t="inlineStr">
@@ -2156,17 +2156,17 @@
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>La Asamblea Ciudadana Itinerante del Concejo de Bogotá es una iniciativa de participación ciudadana deliberativa que ha tenido lugar en varias ocasiones desde 2020. Organizada por el Concejo de Bogotá y su laboratorio de innovación pública, DemoLab, con el apoyo de organizaciones como iDeemos y la Fundación Avina, esta asamblea busca involucrar a la ciudadanía en la discusión y formulación de políticas públicas sobre temas clave para la ciudad, como movilidad, seguridad, ambiente y ordenamiento territorial (Año: 2020).</t>
+          <t>La Plataforma UCampus fue la herramienta digital oficial utilizada en el proceso constituyente de Chile en 2023, desarrollada por el Centro Tecnológico UCampus de la Facultad de Ciencias Físicas y Matemáticas de la Universidad de Chile. Su objetivo principal fue facilitar la participación ciudadana en la redacción de una nueva Constitución, ofreciendo un espacio accesible y seguro para que la ciudadanía pudiera involucrarse activamente en este proceso histórico (Año: 2023-24).</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>https://concejodebogota.gov.co/llega-al-concejo-de-bogota-la-tercera-asamblea-ciudadana-que-busca/cbogota/2023-05-23/084537.php</t>
+          <t>https://ucampus.cl/ucampus-es-la-plataforma-digital-del-proceso-constitucional-2023/</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: El proceso es elegible en su forma (mini-publico deliberativo recurrente convocado por gobierno local: Concejo de Bogota via DemoLab; 3 ediciones 2020/2021/2023). Sin embargo, NO se encontro evidencia de uso de inteligencia artificial sobre el CONTENIDO de los aportes ciudadanos dentro del proceso participativo en ninguna de sus ediciones → se confirma el motivo de exclusión 2025 → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (concejodebogota.gov.co)]</t>
+          <t>Motivo 2025: «No evidencia de uso de IA» · Reconfirmación 2026: MANTENER EXCLUIDO. Existe un proceso participativo ELEGIBLE (Proceso Constitucional 2023, mecanismos de participación ciudadana con ~280 mil personas, convocado por el Estado de Chile), y UCampus (Universidad de Chile) fue el operador técnico de dos de los cuatro mecanismos (Audiencias Públicas e Iniciativa Popular de Norma), pero no se encontró evidencia de que se aplicara IA/NLP sobre el CONTENIDO de los aportes en esos mecanismos → el motivo 2025 («No evidencia de uso de IA») sigue vigente → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv (por qué se revisó) y URL del caso (ucampus.cl)]</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>Chatbot ALBA</t>
+          <t>Asamblea Ciudadana Itinerante del Concejo de Bogotá</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
@@ -2188,17 +2188,17 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Asistente virtual de la Alcaldía de Barranquilla que facilita información sobre trámites y servicios (Año: 2021).</t>
+          <t>La Asamblea Ciudadana Itinerante del Concejo de Bogotá es una iniciativa de participación ciudadana deliberativa que ha tenido lugar en varias ocasiones desde 2020. Organizada por el Concejo de Bogotá y su laboratorio de innovación pública, DemoLab, con el apoyo de organizaciones como iDeemos y la Fundación Avina, esta asamblea busca involucrar a la ciudadanía en la discusión y formulación de políticas públicas sobre temas clave para la ciudad, como movilidad, seguridad, ambiente y ordenamiento territorial (Año: 2020).</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>https://barranquilla.gov.co/chatbot</t>
+          <t>https://concejodebogota.gov.co/llega-al-concejo-de-bogota-la-tercera-asamblea-ciudadana-que-busca/cbogota/2023-05-23/084537.php</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: El proceso es elegible en su forma (mini-publico deliberativo recurrente convocado por gobierno local: Concejo de Bogota via DemoLab; 3 ediciones 2020/2021/2023). Sin embargo, NO se encontro evidencia de uso de inteligencia artificial sobre el CONTENIDO de los aportes ciudadanos dentro del proceso participativo en ninguna de sus ediciones → se confirma el motivo de exclusión 2025 → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (concejodebogota.gov.co)]</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>Chatbot Rama Judicial</t>
+          <t>Chatbot ALBA</t>
         </is>
       </c>
       <c r="C56" s="12" t="inlineStr">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Este chatbot es un software que emplea IA para mantener conversaciones en tiempo real mediante texto con los usuarios. Está diseñado para proporcionar información de primer nivel relacionada con los servicios que ofrece la Rama Judicial, incluyendo detalles de contacto a nivel nacional de direcciones y consejos seccionales. Además, puede redirigir solicitudes al interior de la Rama Judicial y a otras entidades pertinentes (Año: 2024).</t>
+          <t>Asistente virtual de la Alcaldía de Barranquilla que facilita información sobre trámites y servicios (Año: 2021).</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>https://www.ramajudicial.gov.co/web/centro-de-documentacion-judicial/nuevo-chatbot</t>
+          <t>https://barranquilla.gov.co/chatbot</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>Chatbot Rebecca</t>
+          <t>Chatbot Rama Judicial</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
@@ -2252,17 +2252,17 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Rebeca es un Chatbot diseñado para mejorar la interacción entre la ciudadanía y RenoBo, proporcionando respuestas automáticas e inteligentes sobre servicios, trámites y proyectos de la entidad. Al estar disponible las 24 horas del día, y al utilizar procesamiento de lenguaje natural para comprender y responder de manera conversacional, Rebeca facilita que los ciudadanos accedan a información relevante de manera eficiente y personalizada (Año: 2024).</t>
+          <t>Este chatbot es un software que emplea IA para mantener conversaciones en tiempo real mediante texto con los usuarios. Está diseñado para proporcionar información de primer nivel relacionada con los servicios que ofrece la Rama Judicial, incluyendo detalles de contacto a nivel nacional de direcciones y consejos seccionales. Además, puede redirigir solicitudes al interior de la Rama Judicial y a otras entidades pertinentes (Año: 2024).</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>https://bogota.gov.co/mi-ciudad/habitat/bogota-tiene-chatbot-renobo-que-utiliza-inteligencia-artificial</t>
+          <t>https://www.ramajudicial.gov.co/web/centro-de-documentacion-judicial/nuevo-chatbot</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Mini-Public del diálogo social de la Procuraduría</t>
+          <t>Chatbot Rebecca</t>
         </is>
       </c>
       <c r="C58" s="12" t="inlineStr">
@@ -2284,17 +2284,17 @@
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Ejercicio de deliberación ciudadana realizado en 2020 por la Procuraduría General de la Nación de Colombia. Reunió a cerca de 100 ciudadanos de diferentes regiones del país, seleccionados por sorteo, para discutir temas clave como democracia, diversidad, violencia, retorno al campo y protección social (Año: 2020).</t>
+          <t>Rebeca es un Chatbot diseñado para mejorar la interacción entre la ciudadanía y RenoBo, proporcionando respuestas automáticas e inteligentes sobre servicios, trámites y proyectos de la entidad. Al estar disponible las 24 horas del día, y al utilizar procesamiento de lenguaje natural para comprender y responder de manera conversacional, Rebeca facilita que los ciudadanos accedan a información relevante de manera eficiente y personalizada (Año: 2024).</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>https://ideemos.org/mini-public-del-dialogo-social-de-la-procuraduria/</t>
+          <t>https://bogota.gov.co/mi-ciudad/habitat/bogota-tiene-chatbot-renobo-que-utiliza-inteligencia-artificial</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: Se MANTIENE EXCLUIDO (entra=NO), confirmando el motivo de exclusión de 2025 ('No se encontró información sobre el uso de la IA en la implementación de los Mini Publics'). El proceso es ELEGIBLE por su naturaleza (mini-público / diálogo social deliberativo convocado por la Procuraduría General de la Nación, operado con la metodología de Ideemos), pero sin evidencia de uso de IA sobre el contenido de los aportes → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (ideemos.org)]</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>Pa' que veás (Cali)</t>
+          <t>Mini-Public del diálogo social de la Procuraduría</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
@@ -2316,17 +2316,17 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Conjunto de bots que recopilan quejas y predicen riesgos en obras públicas; tablero abierto (Año: 2025).</t>
+          <t>Ejercicio de deliberación ciudadana realizado en 2020 por la Procuraduría General de la Nación de Colombia. Reunió a cerca de 100 ciudadanos de diferentes regiones del país, seleccionados por sorteo, para discutir temas clave como democracia, diversidad, violencia, retorno al campo y protección social (Año: 2020).</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>https://www.iadb.org/en/news/city-cali-launches-platform-monitoring-public-investment-idb-support</t>
+          <t>https://ideemos.org/mini-public-del-dialogo-social-de-la-procuraduria/</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>Motivo 2025: «No evidencia de uso de IA» · Reconfirmación 2026: Se revisa por su analogia con dIAra (bots que recopilan quejas ciudadanas y predicen riesgos en obras). Sin embargo, NO se encontro evidencia de uso de inteligencia artificial sobre el CONTENIDO de los aportes/quejas ciudadanas dentro de un proceso participativo. 'Pa' que veas' es, en su nucleo, un civic-tech de monitoreo/fiscalización ciudadana de obras públicas (plataforma de la Alcaldía de Cali con apoyo del BID), no un proceso participativo con IA sobre el contenido de los aportes → MANTENER EXCLUIDO (mismo criterio corregido que dejó fuera a dIAra). [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (iadb.org)]</t>
+          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: Se MANTIENE EXCLUIDO (entra=NO), confirmando el motivo de exclusión de 2025 ('No se encontró información sobre el uso de la IA en la implementación de los Mini Publics'). El proceso es ELEGIBLE por su naturaleza (mini-público / diálogo social deliberativo convocado por la Procuraduría General de la Nación, operado con la metodología de Ideemos), pero sin evidencia de uso de IA sobre el contenido de los aportes → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (ideemos.org)]</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Plataforma Urna de Cristal</t>
+          <t>Pa' que veás (Cali)</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Monitorear en tiempo real la opinión ciudadana para ajustar campañas de comunicación y responder preguntas públicas (Año: 2015 –25).</t>
+          <t>Conjunto de bots que recopilan quejas y predicen riesgos en obras públicas; tablero abierto (Año: 2025).</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf</t>
+          <t>https://www.iadb.org/en/news/city-cali-launches-platform-monitoring-public-investment-idb-support</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>No evidencia de uso de IA</t>
+          <t>Motivo 2025: «No evidencia de uso de IA» · Reconfirmación 2026: Se revisa por su analogia con dIAra (bots que recopilan quejas ciudadanas y predicen riesgos en obras). Sin embargo, NO se encontro evidencia de uso de inteligencia artificial sobre el CONTENIDO de los aportes/quejas ciudadanas dentro de un proceso participativo. 'Pa' que veas' es, en su nucleo, un civic-tech de monitoreo/fiscalización ciudadana de obras públicas (plataforma de la Alcaldía de Cali con apoyo del BID), no un proceso participativo con IA sobre el contenido de los aportes → MANTENER EXCLUIDO (mismo criterio corregido que dejó fuera a dIAra). [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y URL del caso (iadb.org)]</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>SISBÉN IV</t>
+          <t>Plataforma Urna de Cristal</t>
         </is>
       </c>
       <c r="C61" s="12" t="inlineStr">
@@ -2380,17 +2380,17 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Encuesta nacional que, con Quantile Gradient Boosting, clasifica hogares en grupos socio-económicos para asignar subsidios (Año: 2019).</t>
+          <t>Monitorear en tiempo real la opinión ciudadana para ajustar campañas de comunicación y responder preguntas públicas (Año: 2015 –25).</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/sisben</t>
+          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>No evidencia de uso de IA</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
+          <t>SISBÉN IV</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
@@ -2412,29 +2412,29 @@
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Metodología que integra analítica de datos, IA y deliberación ciudadana (mini-publics, jurados, asambleas) para resolver problemas públicos o privados con diálogo informado (Año: 2021).</t>
+          <t>Encuesta nacional que, con Quantile Gradient Boosting, clasifica hogares en grupos socio-económicos para asignar subsidios (Año: 2019).</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>https://ideemos.org/ilabs-laboratorios-de-inteligencia-colectiva/</t>
+          <t>https://fairlac.iadb.org/sisben</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: MANTENER EXCLUIDO. La regla de reingreso exige evidencia de IA aplicada al CONTENIDO de los aportes ciudadanos dentro de un proceso participativo. La fuente primaria (página iLabs de Ideemos y su PDF) describe 'Inteligencia Artificial' y 'Machine Learning' SOLO como parte de un listado de técnicas que su metodología puede integrar, sin evidencia de un despliegue concreto de IA sobre el contenido de los aportes en un proceso participativo específico → se confirma el motivo 2025 → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y PDF de iLabs (URL del caso)]</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>iLabs - Laboratorios de Inteligencia Colectiva (Ideemos)</t>
         </is>
       </c>
       <c r="C63" s="12" t="inlineStr">
@@ -2444,17 +2444,17 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Sara es un chatbot de inteligencia artificial desarrollado por el Programa de las Naciones Unidas para el Desarrollo (PNUD),, con el objetivo de prevenir y atender la violencia de género en Centroamérica y la República Dominicana (Año: 2024-25).</t>
+          <t>Metodología que integra analítica de datos, IA y deliberación ciudadana (mini-publics, jurados, asambleas) para resolver problemas públicos o privados con diálogo informado (Año: 2021).</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
+          <t>https://ideemos.org/ilabs-laboratorios-de-inteligencia-colectiva/</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>Motivo 2025: «No se encontró información sobre el uso de la IA en la implementación de los Mini Publics» · Reconfirmación 2026: MANTENER EXCLUIDO. La regla de reingreso exige evidencia de IA aplicada al CONTENIDO de los aportes ciudadanos dentro de un proceso participativo. La fuente primaria (página iLabs de Ideemos y su PDF) describe 'Inteligencia Artificial' y 'Machine Learning' SOLO como parte de un listado de técnicas que su metodología puede integrar, sin evidencia de un despliegue concreto de IA sobre el contenido de los aportes en un proceso participativo específico → se confirma el motivo 2025 → MANTENER EXCLUIDO. [Cierre reconstruido: el insumo de validación traía este texto truncado a 300 caracteres; fuentes: data/candidatos/excluidos_revisar.csv y PDF de iLabs (URL del caso)]</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>TAÍNA: Gobierno Inteligente</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
@@ -2476,29 +2476,29 @@
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Plataforma de IA conversacional de texto y voz para tramitar servicios públicos y anticipar necesidades ciudadanas, parte de la Estrategia Nacional de Inteligencia Artificial (ENIA) (Año: 2023).</t>
+          <t>Sara es un chatbot de inteligencia artificial desarrollado por el Programa de las Naciones Unidas para el Desarrollo (PNUD),, con el objetivo de prevenir y atender la violencia de género en Centroamérica y la República Dominicana (Año: 2024-25).</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>https://www.diariolibre.com/actualidad/nacional/2023/10/11/gobierno-presenta-estrategia-de-inteligencia-artificial/2489157</t>
+          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>LATAM</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>ANTAI Smart CID (Autoridad Nacional de Transparencia y Acceso a la Información + OS City)</t>
+          <t>TAÍNA: Gobierno Inteligente</t>
         </is>
       </c>
       <c r="C65" s="12" t="inlineStr">
@@ -2508,17 +2508,17 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>CAF invirtió en la startup govtech OS City para acelerar la digitalización de trámites y la emisión de credenciales oficiales con blockchain e IA, impulsando su expansión regional (Año: 2021).</t>
+          <t>Plataforma de IA conversacional de texto y voz para tramitar servicios públicos y anticipar necesidades ciudadanas, parte de la Estrategia Nacional de Inteligencia Artificial (ENIA) (Año: 2023).</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
+          <t>https://www.diariolibre.com/actualidad/nacional/2023/10/11/gobierno-presenta-estrategia-de-inteligencia-artificial/2489157</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>Botivist</t>
+          <t>ANTAI Smart CID (Autoridad Nacional de Transparencia y Acceso a la Información + OS City)</t>
         </is>
       </c>
       <c r="C66" s="12" t="inlineStr">
@@ -2540,17 +2540,17 @@
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Botivist es una iniciativa de Microsoft Research que usa inteligencia artificial para promover la participación ciudadana en causas sociales. Utiliza bots en Twitter que detectan conversaciones sobre temas como corrupción y luego invitan a los usuarios a colaborar en la búsqueda de soluciones. Botivist es una iniciativa desarrollada por investigadores de la Universidad de West Virginia, Microsoft Research y la UNAM, que utiliza inteligencia artificial para fomentar la participación ciudadana a través de Twitter. Emplea bots programados con diferentes estrategias comunicativas para convocar y motivar a voluntarios a colaborar en causas sociales, como la lucha contra la corrupción. La IA se aplica en la identificación de usuarios potencialmente interesados, en el análisis de respuestas y en la adaptación del lenguaje de los bots para maximizar el compromiso. En sus pruebas, Botivist logró que más del 80% de los usuarios que interactuaron con los bots aportaran propuestas útiles, demostrando su eficacia como herramienta digital para la acción colectiva (Año: 2016).</t>
+          <t>CAF invirtió en la startup govtech OS City para acelerar la digitalización de trámites y la emisión de credenciales oficiales con blockchain e IA, impulsando su expansión regional (Año: 2021).</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com/en-us/research/publication/botivist-calling-volunteers-to-action-using-online-bots/</t>
+          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
-          <t>No tiene foco en un país específico</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>Chatbot DCI (Denuncia Ciudadana Idónea)</t>
+          <t>Botivist</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
@@ -2572,17 +2572,17 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Chatbot web que guía a la ciudadanía para formular y encauzar denuncias de corrupción ante las Entidades Fiscalizadoras Superiores (EFS) de los cuatro países participantes (Año: 2024).</t>
+          <t>Botivist es una iniciativa de Microsoft Research que usa inteligencia artificial para promover la participación ciudadana en causas sociales. Utiliza bots en Twitter que detectan conversaciones sobre temas como corrupción y luego invitan a los usuarios a colaborar en la búsqueda de soluciones. Botivist es una iniciativa desarrollada por investigadores de la Universidad de West Virginia, Microsoft Research y la UNAM, que utiliza inteligencia artificial para fomentar la participación ciudadana a través de Twitter. Emplea bots programados con diferentes estrategias comunicativas para convocar y motivar a voluntarios a colaborar en causas sociales, como la lucha contra la corrupción. La IA se aplica en la identificación de usuarios potencialmente interesados, en el análisis de respuestas y en la adaptación del lenguaje de los bots para maximizar el compromiso. En sus pruebas, Botivist logró que más del 80% de los usuarios que interactuaron con los bots aportaran propuestas útiles, demostrando su eficacia como herramienta digital para la acción colectiva (Año: 2016).</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
+          <t>https://www.microsoft.com/en-us/research/publication/botivist-calling-volunteers-to-action-using-online-bots/</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>No evidencia de uso de IA</t>
+          <t>No tiene foco en un país específico</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>Citibeats: Covid-19 (“Percepciones ciudadanas COVID-19”)</t>
+          <t>Chatbot DCI (Denuncia Ciudadana Idónea)</t>
         </is>
       </c>
       <c r="C68" s="12" t="inlineStr">
@@ -2604,17 +2604,17 @@
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Escucha social de opiniones en Twitter y foros para detectar temas, sentimiento y desinformación sobre salud, empleo, educación, etc., generando alertas para ajustar la comunicación pública (Año: 2020).</t>
+          <t>Chatbot web que guía a la ciudadanía para formular y encauzar denuncias de corrupción ante las Entidades Fiscalizadoras Superiores (EFS) de los cuatro países participantes (Año: 2024).</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>https://forbescentroamerica.com/2021/04/28/civiclytics-el-big-data-apoya-la-recuperacion-economica</t>
+          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Análisis de redes sociales, no es participación</t>
+          <t>No evidencia de uso de IA</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>Ushahidi "AI for Good"</t>
+          <t>Citibeats: Covid-19 (“Percepciones ciudadanas COVID-19”)</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
@@ -2636,29 +2636,29 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Es una plataforma digital de código abierto creada en 2008 para recopilar y mapear información enviada por ciudadanos en contextos como elecciones, crisis o desastres. Desde 2023, incorpora inteligencia artificial para clasificar automáticamente reportes, mejorar la geolocalización, traducir textos y detectar duplicados, facilitando así una participación ciudadana más eficiente y una toma de decisiones más informada por parte de gobiernos y organizaciones (Año: 2023).</t>
+          <t>Escucha social de opiniones en Twitter y foros para detectar temas, sentimiento y desinformación sobre salud, empleo, educación, etc., generando alertas para ajustar la comunicación pública (Año: 2020).</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>https://www.ushahidi.com/</t>
+          <t>https://forbescentroamerica.com/2021/04/28/civiclytics-el-big-data-apoya-la-recuperacion-economica</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>No se evidencia el uso de IA en los proyectos de participación listados para Latam</t>
+          <t>Análisis de redes sociales, no es participación</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>LATAM</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>AMIMgo</t>
+          <t>Ushahidi "AI for Good"</t>
         </is>
       </c>
       <c r="C70" s="12" t="inlineStr">
@@ -2668,17 +2668,17 @@
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>AMIMgo, un chatbot de atención ciudadana disponible a través de WhatsApp. Esta herramienta permite a los usuarios reportar y dar seguimiento a incidencias relacionadas con semáforos, señalización vial, infraestructura ciclista y el sistema de bicicletas públicas MiBici (Año: 2023).</t>
+          <t>Es una plataforma digital de código abierto creada en 2008 para recopilar y mapear información enviada por ciudadanos en contextos como elecciones, crisis o desastres. Desde 2023, incorpora inteligencia artificial para clasificar automáticamente reportes, mejorar la geolocalización, traducir textos y detectar duplicados, facilitando así una participación ciudadana más eficiente y una toma de decisiones más informada por parte de gobiernos y organizaciones (Año: 2023).</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>https://amim.mx/noticias/detalle/estrena-amim-chatbot-para-la-atencion-ciudadana</t>
+          <t>https://www.ushahidi.com/</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>No se evidencia el uso de IA en los proyectos de participación listados para Latam</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>ATIC</t>
+          <t>AMIMgo</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
@@ -2700,17 +2700,17 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>ATIC es un chatbot que funciona a través de WhatsApp, así como por medio de una computadora y está entrenado para comprender una amplia gama de preguntas relacionadas al derecho de acceso a la información; obtener detalles sobre el presupuesto público, salarios de los funcionarios, facturas y empresas que intervienen en proyectos dentro de la Ciudad de México (Año: 2024-25).</t>
+          <t>AMIMgo, un chatbot de atención ciudadana disponible a través de WhatsApp. Esta herramienta permite a los usuarios reportar y dar seguimiento a incidencias relacionadas con semáforos, señalización vial, infraestructura ciclista y el sistema de bicicletas públicas MiBici (Año: 2023).</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>https://oem.com.mx/la-prensa/metropoli/info-cdmx-implementa-atic-una-herramienta-con-ia-que-facilita-el-acceso-a-la-informacion-13081722</t>
+          <t>https://amim.mx/noticias/detalle/estrena-amim-chatbot-para-la-atencion-ciudadana</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="B72" s="9" t="inlineStr">
         <is>
-          <t>ChatBot “Claudia"</t>
+          <t>ATIC</t>
         </is>
       </c>
       <c r="C72" s="12" t="inlineStr">
@@ -2732,17 +2732,17 @@
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Chatbot generativo que combina GPT-4 con recuperación aumentada de información sobre más de 1000 discursos, artículos y debates de Claudia Sheinbaum. Responde preguntas del público emulando su tono y razonamiento técnico para dialogar sobre transición energética, cambio climático y política pública, fomentando un debate ciudadano informado (Año: 2024).</t>
+          <t>ATIC es un chatbot que funciona a través de WhatsApp, así como por medio de una computadora y está entrenado para comprender una amplia gama de preguntas relacionadas al derecho de acceso a la información; obtener detalles sobre el presupuesto público, salarios de los funcionarios, facturas y empresas que intervienen en proyectos dentro de la Ciudad de México (Año: 2024-25).</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>https://mexicocomovamos.mx/animal-politico/2024/08/chatbot-claudia-una-herramienta-de-participacion-ciudadana/</t>
+          <t>https://oem.com.mx/la-prensa/metropoli/info-cdmx-implementa-atic-una-herramienta-con-ia-que-facilita-el-acceso-a-la-informacion-13081722</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
         <is>
-          <t>No es participación</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B73" s="9" t="inlineStr">
         <is>
-          <t>Chatbot "Inés"</t>
+          <t>ChatBot “Claudia"</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
@@ -2764,17 +2764,17 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Chatbot en WhatsApp que brinda información electoral y permite verificar la veracidad de contenidos relacionados con las elecciones (Año: 2021).</t>
+          <t>Chatbot generativo que combina GPT-4 con recuperación aumentada de información sobre más de 1000 discursos, artículos y debates de Claudia Sheinbaum. Responde preguntas del público emulando su tono y razonamiento técnico para dialogar sobre transición energética, cambio climático y política pública, fomentando un debate ciudadano informado (Año: 2024).</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>https://centralelectoral.ine.mx/2024/04/17/nueva-version-del-chatbot-del-ine-en-whatsapp-permitira-verificar-informacion-sobre-elecciones-2024/</t>
+          <t>https://mexicocomovamos.mx/animal-politico/2024/08/chatbot-claudia-una-herramienta-de-participacion-ciudadana/</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>No es participación, es informativo</t>
+          <t>No es participación</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B74" s="9" t="inlineStr">
         <is>
-          <t>Chatbot Sam Petrino</t>
+          <t>Chatbot "Inés"</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
@@ -2796,17 +2796,17 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Chatbot desarrollado por Cívica Digital e implementado en San Pedro Garza García en febrero de 2020, un mes antes del inicio de la pandemia, como única vía de comunicación entre la ciudadanía y el gobierno municipal a través de WhatsApp y Facebook Chat. Inicialmente concebido para reportes de servicios públicos (luminarias, baches, recolección de basura, etc.) (Año: 2020).</t>
+          <t>Chatbot en WhatsApp que brinda información electoral y permite verificar la veracidad de contenidos relacionados con las elecciones (Año: 2021).</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>https://www.civica.digital/historias/chatbot-sam-petrino</t>
+          <t>https://centralelectoral.ine.mx/2024/04/17/nueva-version-del-chatbot-del-ine-en-whatsapp-permitira-verificar-informacion-sobre-elecciones-2024/</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación, es informativo</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B75" s="9" t="inlineStr">
         <is>
-          <t>Chatbot Victoria</t>
+          <t>Chatbot Sam Petrino</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Chatbot para ayudar a los ciudadanos a mantenerse informados y seguros durante la pandemia por Covid-19. Este servicio, disponible en redes sociales desde el 2019 para brindar información general sobre la ciudad, ahora en su versión para WhatsApp incorporó información oficial y confiable sobre la enfermedad y su propagación; datos sobre la capacidad hospitalaria en la ciudad; y una asesoría rápida las 24 horas del día para determinar si un caso requería de atención médica (Año: 2019-25).</t>
+          <t>Chatbot desarrollado por Cívica Digital e implementado en San Pedro Garza García en febrero de 2020, un mes antes del inicio de la pandemia, como única vía de comunicación entre la ciudadanía y el gobierno municipal a través de WhatsApp y Facebook Chat. Inicialmente concebido para reportes de servicios públicos (luminarias, baches, recolección de basura, etc.) (Año: 2020).</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>https://adip.cdmx.gob.mx/comunicacion/nota/la-adip-y-el-gobierno-de-la-ciudad-presentan-victoria-el-robot-que-colaborara-en-la-atencion-de-la-ciudadania</t>
+          <t>https://www.civica.digital/historias/chatbot-sam-petrino</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>INAOE (Conacyt) – Laboratorio de Tecnologías del Lenguaje</t>
+          <t>Chatbot Victoria</t>
         </is>
       </c>
       <c r="C76" s="12" t="inlineStr">
@@ -2860,17 +2860,17 @@
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Algoritmos que analizan grandes volúmenes de texto en redes sociales para detectar indicios de depresión, anorexia u otros trastornos mentales en la población, con el fin de fundamentar políticas públicas de salud y asistir a quienes lo necesitenoecd.orgoecd.org (Año: 2018–25 ).</t>
+          <t>Chatbot para ayudar a los ciudadanos a mantenerse informados y seguros durante la pandemia por Covid-19. Este servicio, disponible en redes sociales desde el 2019 para brindar información general sobre la ciudad, ahora en su versión para WhatsApp incorporó información oficial y confiable sobre la enfermedad y su propagación; datos sobre la capacidad hospitalaria en la ciudad; y una asesoría rápida las 24 horas del día para determinar si un caso requería de atención médica (Año: 2019-25).</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://adip.cdmx.gob.mx/comunicacion/nota/la-adip-y-el-gobierno-de-la-ciudad-presentan-victoria-el-robot-que-colaborara-en-la-atencion-de-la-ciudadania</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>Movimex</t>
+          <t>INAOE (Conacyt) – Laboratorio de Tecnologías del Lenguaje</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
@@ -2892,12 +2892,12 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>El Chatbot MOVIMEX es una herramienta digital implementada por la Secretaría de Movilidad del Estado de México (Semov) en colaboración con Meta, que permite a los ciudadanos realizar trámites y presentar denuncias relacionadas con la movilidad a través de WhatsApp (Año: 2024).</t>
+          <t>Algoritmos que analizan grandes volúmenes de texto en redes sociales para detectar indicios de depresión, anorexia u otros trastornos mentales en la población, con el fin de fundamentar políticas públicas de salud y asistir a quienes lo necesitenoecd.orgoecd.org (Año: 2018–25 ).</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>https://animalpolitico.com/estados/chatbot-movimex-tramites-denuncias-edomex</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>Sistema *0311 Locatel</t>
+          <t>Movimex</t>
         </is>
       </c>
       <c r="C78" s="12" t="inlineStr">
@@ -2924,17 +2924,17 @@
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Plataforma de atención ciudadana que utiliza IA para clasificar y despachar en tiempo real solicitudes de servicios urbanos y no emergencias, mejorando la eficiencia y tiempos de respuesta del gobierno de la Ciudad de México (Año: 2021).</t>
+          <t>El Chatbot MOVIMEX es una herramienta digital implementada por la Secretaría de Movilidad del Estado de México (Semov) en colaboración con Meta, que permite a los ciudadanos realizar trámites y presentar denuncias relacionadas con la movilidad a través de WhatsApp (Año: 2024).</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>https://research.latinxinai.org/papers/naacl/2022/pdf/paper_01.pdf</t>
+          <t>https://animalpolitico.com/estados/chatbot-movimex-tramites-denuncias-edomex</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Atención ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>Violetta</t>
+          <t>Sistema *0311 Locatel</t>
         </is>
       </c>
       <c r="C79" s="12" t="inlineStr">
@@ -2956,29 +2956,29 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>Plataforma digital que mediante un chatbot con inteligencia artificial, ofrece de forma gratuita, inmediata y recurrente recursos psicoeducativos para prevenir la violencia de género y fomentar relaciones sanas. Su misión es convertirse en la plataforma sostenible y multidisciplinaria líder, proporcionando tecnologías escalables y expertos que guíen a las personas hacia relaciones libres de violencia (Año: 2023-25).</t>
+          <t>Plataforma de atención ciudadana que utiliza IA para clasificar y despachar en tiempo real solicitudes de servicios urbanos y no emergencias, mejorando la eficiencia y tiempos de respuesta del gobierno de la Ciudad de México (Año: 2021).</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>https://holasoyvioletta.com/acerca-de/</t>
+          <t>https://research.latinxinai.org/papers/naacl/2022/pdf/paper_01.pdf</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>Atención ciudadana</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>Dr. ROSA y Dr. NICO</t>
+          <t>Violetta</t>
         </is>
       </c>
       <c r="C80" s="12" t="inlineStr">
@@ -2988,29 +2988,29 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Amplio uso durante la pandemia para evaluación temprana de casos. Facilitó la detección y canalización de pacientes COVID, reduciendo la carga en centros de salud. Reconocido como ejemplo regional de IA aplicada a emergencias sanitariasoecd.orgoecd.org (Año: 2020).</t>
+          <t>Plataforma digital que mediante un chatbot con inteligencia artificial, ofrece de forma gratuita, inmediata y recurrente recursos psicoeducativos para prevenir la violencia de género y fomentar relaciones sanas. Su misión es convertirse en la plataforma sostenible y multidisciplinaria líder, proporcionando tecnologías escalables y expertos que guíen a las personas hacia relaciones libres de violencia (Año: 2023-25).</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://holasoyvioletta.com/acerca-de/</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>No es participación ciudadana</t>
+          <t>Atencion ciudadana</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr">
         <is>
-          <t>JNE WhatsApp Chatbot</t>
+          <t>Dr. ROSA y Dr. NICO</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
@@ -3020,12 +3020,12 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Permite consultar CV y antecedentes de candidatos y reporte de irregularidades (Año: 2020-25).</t>
+          <t>Amplio uso durante la pandemia para evaluación temprana de casos. Facilitó la detección y canalización de pacientes COVID, reduciendo la carga en centros de salud. Reconocido como ejemplo regional de IA aplicada a emergencias sanitariasoecd.orgoecd.org (Año: 2020).</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>https://portal.jne.gob.pe/Portal/Pagina/Nota/12783</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
@@ -3037,12 +3037,12 @@
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>PY</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>ParaEmpleo</t>
+          <t>JNE WhatsApp Chatbot</t>
         </is>
       </c>
       <c r="C82" s="12" t="inlineStr">
@@ -3052,12 +3052,12 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Recomendador de ofertas y capacitaciones que alinea CV con demanda empresarial (Año: 2019-25).</t>
+          <t>Permite consultar CV y antecedentes de candidatos y reporte de irregularidades (Año: 2020-25).</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/en/paraempleo</t>
+          <t>https://portal.jne.gob.pe/Portal/Pagina/Nota/12783</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
@@ -3069,12 +3069,12 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>UY</t>
+          <t>PY</t>
         </is>
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>Chatbot (Asistente virtual entrenado con IA)</t>
+          <t>ParaEmpleo</t>
         </is>
       </c>
       <c r="C83" s="12" t="inlineStr">
@@ -3084,17 +3084,17 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Asistente Virtual de AGESIC – Chatbot gubernamental piloto lanzado en 2018 para adquirir experiencia en soluciones de IA en la atención ciudadana. Entrenado con preguntas frecuentes recibidas en los distintos canales de contacto del Estadooecd.org. No solo contesta consultas de trámites, sino que puede ejecutar acciones (ej. reestablecer contraseña de usuario) para resolver problemas comunesoecd.org. Integrado en la estrategia multicanal de atención, buscando acercar el Estado a la gente eliminando barreras de acceso (Año: 2018–25).</t>
+          <t>Recomendador de ofertas y capacitaciones que alinea CV con demanda empresarial (Año: 2019-25).</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+          <t>https://fairlac.iadb.org/en/paraempleo</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Atencion ciudadana</t>
+          <t>No es participación ciudadana</t>
         </is>
       </c>
     </row>
@@ -3106,32 +3106,64 @@
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
+          <t>Chatbot (Asistente virtual entrenado con IA)</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>Base 2025 — ya estaba EXCLUIDO, exclusión reconfirmada</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Asistente Virtual de AGESIC – Chatbot gubernamental piloto lanzado en 2018 para adquirir experiencia en soluciones de IA en la atención ciudadana. Entrenado con preguntas frecuentes recibidas en los distintos canales de contacto del Estadooecd.org. No solo contesta consultas de trámites, sino que puede ejecutar acciones (ej. reestablecer contraseña de usuario) para resolver problemas comunesoecd.org. Integrado en la estrategia multicanal de atención, buscando acercar el Estado a la gente eliminando barreras de acceso (Año: 2018–25).</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>Atencion ciudadana</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>UY</t>
+        </is>
+      </c>
+      <c r="B85" s="9" t="inlineStr">
+        <is>
           <t>Consulta Pública de la Estrategia Nacional de Inteligencia Artificial (IA) de Uruguay 2024–2030,</t>
         </is>
       </c>
-      <c r="C84" s="12" t="inlineStr">
-        <is>
-          <t>Base 2025 — ya estaba EXCLUIDO, exclusión reconfirmada</t>
-        </is>
-      </c>
-      <c r="D84" s="9" t="inlineStr">
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>Base 2025 — ya estaba EXCLUIDO, exclusión reconfirmada</t>
+        </is>
+      </c>
+      <c r="D85" s="9" t="inlineStr">
         <is>
           <t>Es una iniciativa del gobierno uruguayo para definir una política pública de IA que abarque los sectores público, privado, académico y de la sociedad civil. Su objetivo es fomentar el desarrollo y uso ético, responsable y seguro de la IA, promoviendo el crecimiento económico inclusivo, la sostenibilidad ambiental y el fortalecimiento de la soberanía nacional (Año: 2024).</t>
         </is>
       </c>
-      <c r="E84" s="9" t="inlineStr">
+      <c r="E85" s="9" t="inlineStr">
         <is>
           <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030</t>
         </is>
       </c>
-      <c r="F84" s="9" t="inlineStr">
+      <c r="F85" s="9" t="inlineStr">
         <is>
           <t>No evidencia de uso de IA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F84"/>
+  <autoFilter ref="A5:F85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>